<commit_message>
feat: partner_short 필드 추가 + contact channel 선택화 + 상품 테이블 파트너 컬럼 개선
- products.partner_short 컬럼 지원 (ProductForm 입력 필드, Excel upload 파싱, diff 감지)
- 카탈로그 filter pills (admin/agent) 및 agent 카드 eyebrow에 partner_short ?? partner_name 적용
- admin products 테이블: Partner 컬럼을 Product Name 왼쪽으로 이동, partner_short 표시
- contact channel 필수 조건 제거 (선택 필드로 변경)
- 5/13 연구노트 업데이트

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/products_master_Hong_260513_K_Beauty 수정_v2.xlsx
+++ b/data/products_master_Hong_260513_K_Beauty 수정_v2.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFD78AC3-835F-4230-B041-95F3FFE991A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA22472D-A9D0-4CD5-A3E5-44796022BD60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="K-Medical" sheetId="1" r:id="rId1"/>
@@ -4151,7 +4151,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AD11"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
@@ -4180,7 +4180,7 @@
     <col min="30" max="30" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:30" s="1" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4272,7 +4272,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:30" s="2" customFormat="1" ht="365.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:30" s="2" customFormat="1" ht="365.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="2" t="s">
         <v>30</v>
       </c>
@@ -4364,7 +4364,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="3" spans="1:30" s="2" customFormat="1" ht="366" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:30" s="2" customFormat="1" ht="366" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A3" s="2" t="s">
         <v>41</v>
       </c>
@@ -4456,7 +4456,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="4" spans="1:30" s="2" customFormat="1" ht="177" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:30" s="2" customFormat="1" ht="177" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A4" s="2" t="s">
         <v>43</v>
       </c>
@@ -4548,7 +4548,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="5" spans="1:30" s="2" customFormat="1" ht="177" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:30" s="2" customFormat="1" ht="177" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A5" s="2" t="s">
         <v>851</v>
       </c>
@@ -4625,7 +4625,7 @@
       </c>
       <c r="AC5" s="3"/>
     </row>
-    <row r="6" spans="1:30" s="2" customFormat="1" ht="177" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:30" s="2" customFormat="1" ht="177" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A6" s="2" t="s">
         <v>852</v>
       </c>
@@ -4702,7 +4702,7 @@
       </c>
       <c r="AC6" s="3"/>
     </row>
-    <row r="7" spans="1:30" s="2" customFormat="1" ht="409.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:30" s="2" customFormat="1" ht="409.6" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A7" s="2" t="s">
         <v>49</v>
       </c>
@@ -4770,7 +4770,7 @@
       </c>
       <c r="AC7" s="3"/>
     </row>
-    <row r="8" spans="1:30" s="2" customFormat="1" ht="409.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:30" s="2" customFormat="1" ht="409.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A8" s="2" t="s">
         <v>50</v>
       </c>
@@ -4838,7 +4838,7 @@
       </c>
       <c r="AC8" s="3"/>
     </row>
-    <row r="9" spans="1:30" s="2" customFormat="1" ht="193.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:30" s="2" customFormat="1" ht="193.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A9" s="2" t="s">
         <v>51</v>
       </c>
@@ -4915,7 +4915,7 @@
       </c>
       <c r="AC9" s="3"/>
     </row>
-    <row r="10" spans="1:30" s="2" customFormat="1" ht="188.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:30" s="2" customFormat="1" ht="188.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A10" s="2" t="s">
         <v>52</v>
       </c>
@@ -4992,7 +4992,7 @@
       </c>
       <c r="AC10" s="3"/>
     </row>
-    <row r="11" spans="1:30" s="2" customFormat="1" ht="177" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:30" s="2" customFormat="1" ht="177" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A11" s="2" t="s">
         <v>53</v>
       </c>
@@ -5084,7 +5084,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:AD23"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
@@ -5113,7 +5113,7 @@
     <col min="30" max="30" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:30" s="1" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -5205,7 +5205,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:30" s="2" customFormat="1" ht="148.5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:30" s="2" customFormat="1" ht="156.6" x14ac:dyDescent="0.4">
       <c r="A2" s="2" t="s">
         <v>876</v>
       </c>
@@ -5288,7 +5288,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="3" spans="1:30" s="2" customFormat="1" ht="132" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:30" s="2" customFormat="1" ht="139.19999999999999" x14ac:dyDescent="0.4">
       <c r="A3" s="2" t="s">
         <v>157</v>
       </c>
@@ -5371,7 +5371,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="4" spans="1:30" s="2" customFormat="1" ht="132" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:30" s="2" customFormat="1" ht="139.19999999999999" x14ac:dyDescent="0.4">
       <c r="A4" s="2" t="s">
         <v>159</v>
       </c>
@@ -5454,7 +5454,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="5" spans="1:30" s="2" customFormat="1" ht="178.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:30" s="2" customFormat="1" ht="178.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A5" s="2" t="s">
         <v>162</v>
       </c>
@@ -5534,7 +5534,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="6" spans="1:30" s="2" customFormat="1" ht="162.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:30" s="2" customFormat="1" ht="162.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A6" s="2" t="s">
         <v>164</v>
       </c>
@@ -5614,7 +5614,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="7" spans="1:30" s="2" customFormat="1" ht="147" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:30" s="2" customFormat="1" ht="147" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A7" s="2" t="s">
         <v>165</v>
       </c>
@@ -5694,7 +5694,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="8" spans="1:30" s="2" customFormat="1" ht="132" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:30" s="2" customFormat="1" ht="139.19999999999999" x14ac:dyDescent="0.4">
       <c r="A8" s="2" t="s">
         <v>167</v>
       </c>
@@ -5777,7 +5777,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="9" spans="1:30" s="2" customFormat="1" ht="214.5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:30" s="2" customFormat="1" ht="208.8" x14ac:dyDescent="0.4">
       <c r="A9" s="2" t="s">
         <v>168</v>
       </c>
@@ -5863,7 +5863,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="10" spans="1:30" s="2" customFormat="1" ht="198" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:30" s="2" customFormat="1" ht="208.8" x14ac:dyDescent="0.4">
       <c r="A10" s="2" t="s">
         <v>169</v>
       </c>
@@ -5949,7 +5949,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="11" spans="1:30" s="2" customFormat="1" ht="132" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:30" s="2" customFormat="1" ht="139.19999999999999" x14ac:dyDescent="0.4">
       <c r="A11" s="2" t="s">
         <v>172</v>
       </c>
@@ -6035,7 +6035,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="12" spans="1:30" s="2" customFormat="1" ht="122.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:30" s="2" customFormat="1" ht="122.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A12" s="2" t="s">
         <v>175</v>
       </c>
@@ -6121,7 +6121,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="13" spans="1:30" s="2" customFormat="1" ht="132" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:30" s="2" customFormat="1" ht="139.19999999999999" x14ac:dyDescent="0.4">
       <c r="A13" s="2" t="s">
         <v>178</v>
       </c>
@@ -6207,7 +6207,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="14" spans="1:30" s="2" customFormat="1" ht="148.5" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:30" s="2" customFormat="1" ht="156.6" x14ac:dyDescent="0.4">
       <c r="A14" s="2" t="s">
         <v>179</v>
       </c>
@@ -6293,7 +6293,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="15" spans="1:30" s="2" customFormat="1" ht="158.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:30" s="2" customFormat="1" ht="158.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A15" s="2" t="s">
         <v>182</v>
       </c>
@@ -6379,7 +6379,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="16" spans="1:30" s="2" customFormat="1" ht="126.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:30" s="2" customFormat="1" ht="126.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A16" s="2" t="s">
         <v>186</v>
       </c>
@@ -6462,7 +6462,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="17" spans="1:29" s="2" customFormat="1" ht="115.5" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:29" s="2" customFormat="1" ht="121.8" x14ac:dyDescent="0.4">
       <c r="A17" s="2" t="s">
         <v>188</v>
       </c>
@@ -6542,7 +6542,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="18" spans="1:29" s="2" customFormat="1" ht="115.5" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:29" s="2" customFormat="1" ht="121.8" x14ac:dyDescent="0.4">
       <c r="A18" s="2" t="s">
         <v>191</v>
       </c>
@@ -6622,35 +6622,35 @@
         <v>200</v>
       </c>
     </row>
-    <row r="19" spans="1:29" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:29" s="2" customFormat="1" x14ac:dyDescent="0.4">
       <c r="F19" s="3"/>
       <c r="P19" s="3"/>
       <c r="Q19" s="3"/>
       <c r="R19" s="3"/>
       <c r="AC19" s="3"/>
     </row>
-    <row r="20" spans="1:29" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:29" s="2" customFormat="1" x14ac:dyDescent="0.4">
       <c r="F20" s="3"/>
       <c r="P20" s="3"/>
       <c r="Q20" s="3"/>
       <c r="R20" s="3"/>
       <c r="AC20" s="3"/>
     </row>
-    <row r="21" spans="1:29" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:29" s="2" customFormat="1" x14ac:dyDescent="0.4">
       <c r="F21" s="3"/>
       <c r="P21" s="3"/>
       <c r="Q21" s="3"/>
       <c r="R21" s="3"/>
       <c r="AC21" s="3"/>
     </row>
-    <row r="22" spans="1:29" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:29" s="2" customFormat="1" x14ac:dyDescent="0.4">
       <c r="F22" s="3"/>
       <c r="P22" s="3"/>
       <c r="Q22" s="3"/>
       <c r="R22" s="3"/>
       <c r="AC22" s="3"/>
     </row>
-    <row r="23" spans="1:29" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:29" s="2" customFormat="1" x14ac:dyDescent="0.4">
       <c r="F23" s="3"/>
       <c r="P23" s="3"/>
       <c r="Q23" s="3"/>
@@ -6667,7 +6667,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:AD77"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
@@ -6696,7 +6696,7 @@
     <col min="30" max="30" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:30" s="1" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -6788,7 +6788,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:30" s="2" customFormat="1" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A2" s="2" t="s">
         <v>907</v>
       </c>
@@ -6880,7 +6880,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="3" spans="1:30" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:30" s="2" customFormat="1" ht="34.799999999999997" x14ac:dyDescent="0.4">
       <c r="A3" s="2" t="s">
         <v>908</v>
       </c>
@@ -6972,7 +6972,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="4" spans="1:30" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:30" s="2" customFormat="1" ht="34.799999999999997" x14ac:dyDescent="0.4">
       <c r="A4" s="2" t="s">
         <v>909</v>
       </c>
@@ -7064,7 +7064,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="5" spans="1:30" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:30" s="2" customFormat="1" ht="34.799999999999997" x14ac:dyDescent="0.4">
       <c r="A5" s="2" t="s">
         <v>910</v>
       </c>
@@ -7156,7 +7156,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:30" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:30" s="2" customFormat="1" ht="34.799999999999997" x14ac:dyDescent="0.4">
       <c r="A6" s="2" t="s">
         <v>911</v>
       </c>
@@ -7248,7 +7248,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="7" spans="1:30" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:30" s="2" customFormat="1" ht="34.799999999999997" x14ac:dyDescent="0.4">
       <c r="A7" s="2" t="s">
         <v>912</v>
       </c>
@@ -7340,7 +7340,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="8" spans="1:30" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:30" s="2" customFormat="1" ht="34.799999999999997" x14ac:dyDescent="0.4">
       <c r="A8" s="2" t="s">
         <v>913</v>
       </c>
@@ -7432,7 +7432,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="9" spans="1:30" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:30" s="2" customFormat="1" ht="34.799999999999997" x14ac:dyDescent="0.4">
       <c r="A9" s="2" t="s">
         <v>914</v>
       </c>
@@ -7524,7 +7524,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="10" spans="1:30" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:30" s="2" customFormat="1" ht="34.799999999999997" x14ac:dyDescent="0.4">
       <c r="A10" s="2" t="s">
         <v>915</v>
       </c>
@@ -7616,7 +7616,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="11" spans="1:30" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:30" s="2" customFormat="1" ht="34.799999999999997" x14ac:dyDescent="0.4">
       <c r="A11" s="2" t="s">
         <v>916</v>
       </c>
@@ -7708,7 +7708,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="12" spans="1:30" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:30" s="2" customFormat="1" ht="34.799999999999997" x14ac:dyDescent="0.4">
       <c r="A12" s="2" t="s">
         <v>917</v>
       </c>
@@ -7800,7 +7800,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="13" spans="1:30" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:30" s="2" customFormat="1" ht="34.799999999999997" x14ac:dyDescent="0.4">
       <c r="A13" s="2" t="s">
         <v>918</v>
       </c>
@@ -7892,7 +7892,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="14" spans="1:30" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:30" s="2" customFormat="1" ht="34.799999999999997" x14ac:dyDescent="0.4">
       <c r="A14" s="2" t="s">
         <v>919</v>
       </c>
@@ -7984,7 +7984,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="15" spans="1:30" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:30" s="2" customFormat="1" ht="34.799999999999997" x14ac:dyDescent="0.4">
       <c r="A15" s="2" t="s">
         <v>920</v>
       </c>
@@ -8076,7 +8076,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="16" spans="1:30" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:30" s="2" customFormat="1" ht="34.799999999999997" x14ac:dyDescent="0.4">
       <c r="A16" s="2" t="s">
         <v>921</v>
       </c>
@@ -8168,7 +8168,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="17" spans="1:30" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:30" s="2" customFormat="1" ht="34.799999999999997" x14ac:dyDescent="0.4">
       <c r="A17" s="2" t="s">
         <v>922</v>
       </c>
@@ -8260,7 +8260,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="18" spans="1:30" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:30" s="2" customFormat="1" ht="34.799999999999997" x14ac:dyDescent="0.4">
       <c r="A18" s="2" t="s">
         <v>923</v>
       </c>
@@ -8352,7 +8352,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="19" spans="1:30" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:30" s="2" customFormat="1" ht="34.799999999999997" x14ac:dyDescent="0.4">
       <c r="A19" s="2" t="s">
         <v>924</v>
       </c>
@@ -8444,7 +8444,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="20" spans="1:30" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:30" s="2" customFormat="1" ht="34.799999999999997" x14ac:dyDescent="0.4">
       <c r="A20" s="2" t="s">
         <v>925</v>
       </c>
@@ -8536,7 +8536,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="21" spans="1:30" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:30" s="2" customFormat="1" ht="34.799999999999997" x14ac:dyDescent="0.4">
       <c r="A21" s="2" t="s">
         <v>926</v>
       </c>
@@ -8628,7 +8628,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="22" spans="1:30" s="2" customFormat="1" ht="99" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:30" s="2" customFormat="1" ht="104.4" x14ac:dyDescent="0.4">
       <c r="A22" s="2" t="s">
         <v>927</v>
       </c>
@@ -8720,7 +8720,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="23" spans="1:30" s="2" customFormat="1" ht="132" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:30" s="2" customFormat="1" ht="104.4" x14ac:dyDescent="0.4">
       <c r="A23" s="2" t="s">
         <v>928</v>
       </c>
@@ -8812,7 +8812,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="24" spans="1:30" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:30" s="2" customFormat="1" ht="69.599999999999994" x14ac:dyDescent="0.4">
       <c r="A24" s="2" t="s">
         <v>929</v>
       </c>
@@ -8904,7 +8904,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="25" spans="1:30" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:30" s="2" customFormat="1" ht="69.599999999999994" x14ac:dyDescent="0.4">
       <c r="A25" s="2" t="s">
         <v>930</v>
       </c>
@@ -8996,7 +8996,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="26" spans="1:30" s="2" customFormat="1" ht="99" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:30" s="2" customFormat="1" ht="104.4" x14ac:dyDescent="0.4">
       <c r="A26" s="2" t="s">
         <v>931</v>
       </c>
@@ -9088,7 +9088,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="27" spans="1:30" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:30" s="2" customFormat="1" ht="69.599999999999994" x14ac:dyDescent="0.4">
       <c r="A27" s="2" t="s">
         <v>932</v>
       </c>
@@ -9180,7 +9180,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="28" spans="1:30" s="2" customFormat="1" ht="99" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:30" s="2" customFormat="1" ht="104.4" x14ac:dyDescent="0.4">
       <c r="A28" s="2" t="s">
         <v>933</v>
       </c>
@@ -9272,7 +9272,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="29" spans="1:30" s="2" customFormat="1" ht="132" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:30" s="2" customFormat="1" ht="121.8" x14ac:dyDescent="0.4">
       <c r="A29" s="2" t="s">
         <v>934</v>
       </c>
@@ -9364,7 +9364,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="30" spans="1:30" s="2" customFormat="1" ht="82.5" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:30" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.4">
       <c r="A30" s="2" t="s">
         <v>935</v>
       </c>
@@ -9456,7 +9456,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="31" spans="1:30" s="2" customFormat="1" ht="82.5" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:30" s="2" customFormat="1" ht="69.599999999999994" x14ac:dyDescent="0.4">
       <c r="A31" s="2" t="s">
         <v>936</v>
       </c>
@@ -9548,7 +9548,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="32" spans="1:30" s="2" customFormat="1" ht="82.5" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:30" s="2" customFormat="1" ht="69.599999999999994" x14ac:dyDescent="0.4">
       <c r="A32" s="2" t="s">
         <v>937</v>
       </c>
@@ -9640,7 +9640,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="33" spans="1:30" s="2" customFormat="1" ht="82.5" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:30" s="2" customFormat="1" ht="69.599999999999994" x14ac:dyDescent="0.4">
       <c r="A33" s="2" t="s">
         <v>938</v>
       </c>
@@ -9732,7 +9732,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="34" spans="1:30" s="2" customFormat="1" ht="82.5" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:30" s="2" customFormat="1" ht="69.599999999999994" x14ac:dyDescent="0.4">
       <c r="A34" s="2" t="s">
         <v>939</v>
       </c>
@@ -9824,7 +9824,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="35" spans="1:30" s="2" customFormat="1" ht="82.5" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:30" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.4">
       <c r="A35" s="2" t="s">
         <v>207</v>
       </c>
@@ -9916,7 +9916,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="36" spans="1:30" s="2" customFormat="1" ht="99" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:30" s="2" customFormat="1" ht="104.4" x14ac:dyDescent="0.4">
       <c r="A36" s="2" t="s">
         <v>216</v>
       </c>
@@ -10008,7 +10008,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="37" spans="1:30" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:30" s="2" customFormat="1" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A37" s="2" t="s">
         <v>224</v>
       </c>
@@ -10100,7 +10100,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="38" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:30" s="2" customFormat="1" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A38" s="2" t="s">
         <v>226</v>
       </c>
@@ -10192,7 +10192,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="39" spans="1:30" s="2" customFormat="1" ht="82.5" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:30" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.4">
       <c r="A39" s="2" t="s">
         <v>229</v>
       </c>
@@ -10284,7 +10284,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="40" spans="1:30" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:30" s="2" customFormat="1" ht="69.599999999999994" x14ac:dyDescent="0.4">
       <c r="A40" s="2" t="s">
         <v>232</v>
       </c>
@@ -10376,7 +10376,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="41" spans="1:30" s="2" customFormat="1" ht="99" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:30" s="2" customFormat="1" ht="104.4" x14ac:dyDescent="0.4">
       <c r="A41" s="2" t="s">
         <v>235</v>
       </c>
@@ -10468,7 +10468,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="42" spans="1:30" s="2" customFormat="1" ht="82.5" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:30" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.4">
       <c r="A42" s="2" t="s">
         <v>241</v>
       </c>
@@ -10554,7 +10554,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="43" spans="1:30" s="2" customFormat="1" ht="115.5" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:30" s="2" customFormat="1" ht="104.4" x14ac:dyDescent="0.4">
       <c r="A43" s="2" t="s">
         <v>244</v>
       </c>
@@ -10640,7 +10640,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="44" spans="1:30" s="2" customFormat="1" ht="99" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:30" s="2" customFormat="1" ht="104.4" x14ac:dyDescent="0.4">
       <c r="A44" s="2" t="s">
         <v>247</v>
       </c>
@@ -10726,7 +10726,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="45" spans="1:30" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:30" s="2" customFormat="1" ht="69.599999999999994" x14ac:dyDescent="0.4">
       <c r="A45" s="2" t="s">
         <v>254</v>
       </c>
@@ -10812,7 +10812,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="46" spans="1:30" s="2" customFormat="1" ht="115.5" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:30" s="2" customFormat="1" ht="121.8" x14ac:dyDescent="0.4">
       <c r="A46" s="2" t="s">
         <v>257</v>
       </c>
@@ -10904,7 +10904,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="47" spans="1:30" s="2" customFormat="1" ht="82.5" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:30" s="2" customFormat="1" ht="69.599999999999994" x14ac:dyDescent="0.4">
       <c r="A47" s="2" t="s">
         <v>261</v>
       </c>
@@ -10996,7 +10996,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="48" spans="1:30" s="2" customFormat="1" ht="82.5" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:30" s="2" customFormat="1" ht="69.599999999999994" x14ac:dyDescent="0.4">
       <c r="A48" s="2" t="s">
         <v>265</v>
       </c>
@@ -11088,7 +11088,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="49" spans="1:30" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:30" s="2" customFormat="1" ht="69.599999999999994" x14ac:dyDescent="0.4">
       <c r="A49" s="2" t="s">
         <v>269</v>
       </c>
@@ -11180,7 +11180,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="50" spans="1:30" s="2" customFormat="1" ht="82.5" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:30" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.4">
       <c r="A50" s="2" t="s">
         <v>272</v>
       </c>
@@ -11272,7 +11272,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="51" spans="1:30" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:30" s="2" customFormat="1" ht="69.599999999999994" x14ac:dyDescent="0.4">
       <c r="A51" s="2" t="s">
         <v>275</v>
       </c>
@@ -11364,7 +11364,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="52" spans="1:30" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:30" s="2" customFormat="1" ht="69.599999999999994" x14ac:dyDescent="0.4">
       <c r="A52" s="2" t="s">
         <v>278</v>
       </c>
@@ -11456,7 +11456,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="53" spans="1:30" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:30" s="2" customFormat="1" ht="69.599999999999994" x14ac:dyDescent="0.4">
       <c r="A53" s="2" t="s">
         <v>281</v>
       </c>
@@ -11548,7 +11548,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="54" spans="1:30" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:30" s="2" customFormat="1" ht="69.599999999999994" x14ac:dyDescent="0.4">
       <c r="A54" s="2" t="s">
         <v>284</v>
       </c>
@@ -11640,7 +11640,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="55" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:30" s="2" customFormat="1" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A55" s="2" t="s">
         <v>940</v>
       </c>
@@ -11732,7 +11732,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="56" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:30" s="2" customFormat="1" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A56" s="2" t="s">
         <v>941</v>
       </c>
@@ -11824,7 +11824,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="57" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:30" s="2" customFormat="1" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A57" s="2" t="s">
         <v>942</v>
       </c>
@@ -11916,7 +11916,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="58" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:30" s="2" customFormat="1" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A58" s="2" t="s">
         <v>943</v>
       </c>
@@ -12008,7 +12008,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="59" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:30" s="2" customFormat="1" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A59" s="2" t="s">
         <v>944</v>
       </c>
@@ -12100,7 +12100,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="60" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:30" s="2" customFormat="1" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A60" s="2" t="s">
         <v>945</v>
       </c>
@@ -12192,7 +12192,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="61" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:30" s="2" customFormat="1" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A61" s="2" t="s">
         <v>946</v>
       </c>
@@ -12284,7 +12284,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="62" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:30" s="2" customFormat="1" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A62" s="2" t="s">
         <v>947</v>
       </c>
@@ -12376,7 +12376,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="63" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:30" s="2" customFormat="1" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A63" s="2" t="s">
         <v>948</v>
       </c>
@@ -12468,7 +12468,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="64" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:30" s="2" customFormat="1" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A64" s="2" t="s">
         <v>949</v>
       </c>
@@ -12560,7 +12560,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="65" spans="1:30" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:30" s="2" customFormat="1" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A65" s="2" t="s">
         <v>598</v>
       </c>
@@ -12652,7 +12652,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="66" spans="1:30" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:30" s="2" customFormat="1" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A66" s="2" t="s">
         <v>605</v>
       </c>
@@ -12744,7 +12744,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="67" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:30" s="2" customFormat="1" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A67" s="2" t="s">
         <v>609</v>
       </c>
@@ -12836,7 +12836,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="68" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:30" s="2" customFormat="1" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A68" s="2" t="s">
         <v>950</v>
       </c>
@@ -12928,7 +12928,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="69" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:30" s="2" customFormat="1" ht="34.799999999999997" x14ac:dyDescent="0.4">
       <c r="A69" s="2" t="s">
         <v>951</v>
       </c>
@@ -13020,7 +13020,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="70" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:30" s="2" customFormat="1" ht="34.799999999999997" x14ac:dyDescent="0.4">
       <c r="A70" s="2" t="s">
         <v>952</v>
       </c>
@@ -13112,7 +13112,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="71" spans="1:30" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:30" s="2" customFormat="1" ht="34.799999999999997" x14ac:dyDescent="0.4">
       <c r="A71" s="2" t="s">
         <v>953</v>
       </c>
@@ -13204,7 +13204,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="72" spans="1:30" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:30" s="2" customFormat="1" ht="34.799999999999997" x14ac:dyDescent="0.4">
       <c r="A72" s="2" t="s">
         <v>612</v>
       </c>
@@ -13296,7 +13296,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="73" spans="1:30" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:30" s="2" customFormat="1" ht="34.799999999999997" x14ac:dyDescent="0.4">
       <c r="A73" s="2" t="s">
         <v>620</v>
       </c>
@@ -13388,7 +13388,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="74" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:30" s="2" customFormat="1" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A74" s="2" t="s">
         <v>624</v>
       </c>
@@ -13480,7 +13480,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="75" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:30" s="2" customFormat="1" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A75" s="2" t="s">
         <v>630</v>
       </c>
@@ -13572,7 +13572,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="76" spans="1:30" s="2" customFormat="1" ht="115.5" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:30" s="2" customFormat="1" ht="104.4" x14ac:dyDescent="0.4">
       <c r="A76" s="2" t="s">
         <v>646</v>
       </c>
@@ -13664,7 +13664,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="77" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:30" s="2" customFormat="1" ht="34.799999999999997" x14ac:dyDescent="0.4">
       <c r="A77" s="2" t="s">
         <v>656</v>
       </c>
@@ -13766,7 +13766,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:AD4"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
@@ -13795,7 +13795,7 @@
     <col min="30" max="30" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:30" s="1" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -13887,7 +13887,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:30" s="2" customFormat="1" ht="115.5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:30" s="2" customFormat="1" ht="104.4" x14ac:dyDescent="0.4">
       <c r="A2" s="2" t="s">
         <v>954</v>
       </c>
@@ -13973,7 +13973,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="3" spans="1:30" s="2" customFormat="1" ht="115.5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:30" s="2" customFormat="1" ht="121.8" x14ac:dyDescent="0.4">
       <c r="A3" s="2" t="s">
         <v>673</v>
       </c>
@@ -14059,7 +14059,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="4" spans="1:30" s="2" customFormat="1" ht="115.5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:30" s="2" customFormat="1" ht="121.8" x14ac:dyDescent="0.4">
       <c r="A4" s="2" t="s">
         <v>728</v>
       </c>
@@ -14155,7 +14155,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:AD4"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
@@ -14184,7 +14184,7 @@
     <col min="30" max="30" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:30" s="1" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -14276,7 +14276,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:30" s="2" customFormat="1" ht="148.5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:30" s="2" customFormat="1" ht="156.6" x14ac:dyDescent="0.4">
       <c r="A2" s="2" t="s">
         <v>955</v>
       </c>
@@ -14368,7 +14368,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="3" spans="1:30" s="2" customFormat="1" ht="148.5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:30" s="2" customFormat="1" ht="156.6" x14ac:dyDescent="0.4">
       <c r="A3" s="2" t="s">
         <v>581</v>
       </c>
@@ -14460,7 +14460,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="4" spans="1:30" s="2" customFormat="1" ht="132" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:30" s="2" customFormat="1" ht="139.19999999999999" x14ac:dyDescent="0.4">
       <c r="A4" s="2" t="s">
         <v>956</v>
       </c>
@@ -14562,7 +14562,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:AD63"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
@@ -14591,7 +14591,7 @@
     <col min="30" max="30" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:30" s="1" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -14683,7 +14683,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:30" s="2" customFormat="1" ht="99" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:30" s="2" customFormat="1" ht="104.4" x14ac:dyDescent="0.4">
       <c r="A2" s="2" t="s">
         <v>957</v>
       </c>
@@ -14775,7 +14775,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="3" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:30" s="2" customFormat="1" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A3" s="2" t="s">
         <v>958</v>
       </c>
@@ -14867,7 +14867,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="4" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:30" s="2" customFormat="1" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A4" s="2" t="s">
         <v>959</v>
       </c>
@@ -14959,7 +14959,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="5" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:30" s="2" customFormat="1" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A5" s="2" t="s">
         <v>960</v>
       </c>
@@ -15051,7 +15051,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:30" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:30" s="2" customFormat="1" ht="34.799999999999997" x14ac:dyDescent="0.4">
       <c r="A6" s="2" t="s">
         <v>961</v>
       </c>
@@ -15143,7 +15143,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="7" spans="1:30" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:30" s="2" customFormat="1" ht="34.799999999999997" x14ac:dyDescent="0.4">
       <c r="A7" s="2" t="s">
         <v>962</v>
       </c>
@@ -15235,7 +15235,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="8" spans="1:30" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:30" s="2" customFormat="1" ht="34.799999999999997" x14ac:dyDescent="0.4">
       <c r="A8" s="2" t="s">
         <v>963</v>
       </c>
@@ -15327,7 +15327,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="9" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:30" s="2" customFormat="1" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A9" s="2" t="s">
         <v>964</v>
       </c>
@@ -15419,7 +15419,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="10" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:30" s="2" customFormat="1" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A10" s="2" t="s">
         <v>965</v>
       </c>
@@ -15511,7 +15511,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="11" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:30" s="2" customFormat="1" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A11" s="2" t="s">
         <v>966</v>
       </c>
@@ -15603,7 +15603,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="12" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:30" s="2" customFormat="1" ht="34.799999999999997" x14ac:dyDescent="0.4">
       <c r="A12" s="2" t="s">
         <v>967</v>
       </c>
@@ -15695,7 +15695,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="13" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:30" s="2" customFormat="1" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A13" s="2" t="s">
         <v>968</v>
       </c>
@@ -15787,7 +15787,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="14" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:30" s="2" customFormat="1" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A14" s="2" t="s">
         <v>969</v>
       </c>
@@ -15879,7 +15879,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="15" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:30" s="2" customFormat="1" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A15" s="2" t="s">
         <v>970</v>
       </c>
@@ -15971,7 +15971,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="16" spans="1:30" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:30" s="2" customFormat="1" ht="34.799999999999997" x14ac:dyDescent="0.4">
       <c r="A16" s="2" t="s">
         <v>971</v>
       </c>
@@ -16063,7 +16063,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="17" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:30" s="2" customFormat="1" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A17" s="2" t="s">
         <v>972</v>
       </c>
@@ -16155,7 +16155,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="18" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:30" s="2" customFormat="1" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A18" s="2" t="s">
         <v>973</v>
       </c>
@@ -16247,7 +16247,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="19" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:30" s="2" customFormat="1" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A19" s="2" t="s">
         <v>974</v>
       </c>
@@ -16339,7 +16339,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="20" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:30" s="2" customFormat="1" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A20" s="2" t="s">
         <v>975</v>
       </c>
@@ -16431,7 +16431,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="21" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:30" s="2" customFormat="1" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A21" s="2" t="s">
         <v>976</v>
       </c>
@@ -16523,7 +16523,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="22" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:30" s="2" customFormat="1" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A22" s="2" t="s">
         <v>977</v>
       </c>
@@ -16615,7 +16615,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="23" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:30" s="2" customFormat="1" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A23" s="2" t="s">
         <v>978</v>
       </c>
@@ -16707,7 +16707,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="24" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:30" s="2" customFormat="1" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A24" s="2" t="s">
         <v>979</v>
       </c>
@@ -16799,7 +16799,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="25" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:30" s="2" customFormat="1" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A25" s="2" t="s">
         <v>980</v>
       </c>
@@ -16891,7 +16891,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="26" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:30" s="2" customFormat="1" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A26" s="2" t="s">
         <v>981</v>
       </c>
@@ -16983,7 +16983,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="27" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:30" s="2" customFormat="1" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A27" s="2" t="s">
         <v>982</v>
       </c>
@@ -17075,7 +17075,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="28" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:30" s="2" customFormat="1" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A28" s="2" t="s">
         <v>983</v>
       </c>
@@ -17167,7 +17167,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="29" spans="1:30" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:30" s="2" customFormat="1" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A29" s="2" t="s">
         <v>984</v>
       </c>
@@ -17259,7 +17259,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="30" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:30" s="2" customFormat="1" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A30" s="2" t="s">
         <v>985</v>
       </c>
@@ -17351,7 +17351,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="31" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:30" s="2" customFormat="1" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A31" s="2" t="s">
         <v>986</v>
       </c>
@@ -17443,7 +17443,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="32" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:30" s="2" customFormat="1" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A32" s="2" t="s">
         <v>987</v>
       </c>
@@ -17535,7 +17535,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="33" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:30" s="2" customFormat="1" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A33" s="2" t="s">
         <v>988</v>
       </c>
@@ -17627,7 +17627,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="34" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:30" s="2" customFormat="1" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A34" s="2" t="s">
         <v>989</v>
       </c>
@@ -17719,7 +17719,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="35" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:30" s="2" customFormat="1" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A35" s="2" t="s">
         <v>990</v>
       </c>
@@ -17811,7 +17811,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="36" spans="1:30" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:30" s="2" customFormat="1" ht="34.799999999999997" x14ac:dyDescent="0.4">
       <c r="A36" s="2" t="s">
         <v>991</v>
       </c>
@@ -17903,7 +17903,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="37" spans="1:30" s="2" customFormat="1" ht="33" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:30" s="2" customFormat="1" ht="34.799999999999997" x14ac:dyDescent="0.4">
       <c r="A37" s="2" t="s">
         <v>992</v>
       </c>
@@ -17995,7 +17995,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="38" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:30" s="2" customFormat="1" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A38" s="2" t="s">
         <v>993</v>
       </c>
@@ -18087,7 +18087,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="39" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:30" s="2" customFormat="1" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A39" s="2" t="s">
         <v>994</v>
       </c>
@@ -18179,7 +18179,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="40" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:30" s="2" customFormat="1" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A40" s="2" t="s">
         <v>995</v>
       </c>
@@ -18271,7 +18271,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="41" spans="1:30" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:30" s="2" customFormat="1" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A41" s="2" t="s">
         <v>996</v>
       </c>
@@ -18363,7 +18363,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="42" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:30" s="2" customFormat="1" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A42" s="2" t="s">
         <v>997</v>
       </c>
@@ -18455,7 +18455,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="43" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:30" s="2" customFormat="1" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A43" s="2" t="s">
         <v>998</v>
       </c>
@@ -18547,7 +18547,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="44" spans="1:30" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:30" s="2" customFormat="1" ht="69.599999999999994" x14ac:dyDescent="0.4">
       <c r="A44" s="2" t="s">
         <v>999</v>
       </c>
@@ -18639,7 +18639,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="45" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:30" s="2" customFormat="1" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A45" s="2" t="s">
         <v>1000</v>
       </c>
@@ -18731,7 +18731,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="46" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:30" s="2" customFormat="1" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A46" s="2" t="s">
         <v>1001</v>
       </c>
@@ -18823,7 +18823,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="47" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:30" s="2" customFormat="1" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A47" s="2" t="s">
         <v>1002</v>
       </c>
@@ -18915,7 +18915,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="48" spans="1:30" s="2" customFormat="1" ht="82.5" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:30" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.4">
       <c r="A48" s="2" t="s">
         <v>1003</v>
       </c>
@@ -19007,7 +19007,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="49" spans="1:30" s="2" customFormat="1" ht="82.5" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:30" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.4">
       <c r="A49" s="2" t="s">
         <v>1004</v>
       </c>
@@ -19099,7 +19099,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="50" spans="1:30" s="2" customFormat="1" ht="99" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:30" s="2" customFormat="1" ht="87" x14ac:dyDescent="0.4">
       <c r="A50" s="2" t="s">
         <v>1005</v>
       </c>
@@ -19191,7 +19191,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="51" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:30" s="2" customFormat="1" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A51" s="2" t="s">
         <v>1006</v>
       </c>
@@ -19283,7 +19283,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="52" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:30" s="2" customFormat="1" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A52" s="2" t="s">
         <v>1007</v>
       </c>
@@ -19375,7 +19375,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="53" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:30" s="2" customFormat="1" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A53" s="2" t="s">
         <v>1008</v>
       </c>
@@ -19467,7 +19467,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="54" spans="1:30" s="2" customFormat="1" ht="49.5" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:30" s="2" customFormat="1" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A54" s="2" t="s">
         <v>1009</v>
       </c>
@@ -19559,7 +19559,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="55" spans="1:30" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:30" s="2" customFormat="1" ht="69.599999999999994" x14ac:dyDescent="0.4">
       <c r="A55" s="2" t="s">
         <v>1010</v>
       </c>
@@ -19651,7 +19651,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="56" spans="1:30" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:30" s="2" customFormat="1" ht="69.599999999999994" x14ac:dyDescent="0.4">
       <c r="A56" s="2" t="s">
         <v>1011</v>
       </c>
@@ -19743,7 +19743,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="57" spans="1:30" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:30" s="2" customFormat="1" ht="69.599999999999994" x14ac:dyDescent="0.4">
       <c r="A57" s="2" t="s">
         <v>1012</v>
       </c>
@@ -19835,7 +19835,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="58" spans="1:30" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:30" s="2" customFormat="1" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A58" s="2" t="s">
         <v>1013</v>
       </c>
@@ -19927,7 +19927,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="59" spans="1:30" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:30" s="2" customFormat="1" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A59" s="2" t="s">
         <v>1014</v>
       </c>
@@ -20019,7 +20019,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="60" spans="1:30" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:30" s="2" customFormat="1" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A60" s="2" t="s">
         <v>1015</v>
       </c>
@@ -20111,7 +20111,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="61" spans="1:30" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:30" s="2" customFormat="1" ht="69.599999999999994" x14ac:dyDescent="0.4">
       <c r="A61" s="2" t="s">
         <v>1016</v>
       </c>
@@ -20203,7 +20203,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="62" spans="1:30" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:30" s="2" customFormat="1" ht="69.599999999999994" x14ac:dyDescent="0.4">
       <c r="A62" s="2" t="s">
         <v>1017</v>
       </c>
@@ -20295,7 +20295,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="63" spans="1:30" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:30" s="2" customFormat="1" ht="69.599999999999994" x14ac:dyDescent="0.4">
       <c r="A63" s="2" t="s">
         <v>1018</v>
       </c>

</xml_diff>